<commit_message>
updated shopping list to buy on farnell - tps62140 not available anymore, buy on mouser or amazon
</commit_message>
<xml_diff>
--- a/hw/RemBrake/assembly/purchase/components.xlsx
+++ b/hw/RemBrake/assembly/purchase/components.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="74" uniqueCount="74">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="77" uniqueCount="77">
   <si>
     <t xml:space="preserve">Part Number</t>
   </si>
@@ -31,6 +31,12 @@
     <t xml:space="preserve">Line Note</t>
   </si>
   <si>
+    <t xml:space="preserve">component name</t>
+  </si>
+  <si>
+    <t xml:space="preserve">one realization</t>
+  </si>
+  <si>
     <t xml:space="preserve">Main switch (waterproof)</t>
   </si>
   <si>
@@ -52,6 +58,9 @@
     <t xml:space="preserve">TPS62140RGTR</t>
   </si>
   <si>
+    <t xml:space="preserve">buy at mouser.de</t>
+  </si>
+  <si>
     <t xml:space="preserve">Ideal Diode</t>
   </si>
   <si>
@@ -64,22 +73,28 @@
     <t xml:space="preserve">LTC2943IDD#TRPBF</t>
   </si>
   <si>
-    <t xml:space="preserve">Voltage detector</t>
+    <t xml:space="preserve">Voltage detector – th=4V0, no delay</t>
   </si>
   <si>
     <t xml:space="preserve">APX803L-40W5-7</t>
   </si>
   <si>
+    <t xml:space="preserve">Voltage detector – th=2V3, adjustable delay</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BD5223G-1TR</t>
+  </si>
+  <si>
     <t xml:space="preserve">555 casovac THT</t>
   </si>
   <si>
-    <t xml:space="preserve">LM555CN/NOPB</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Buzzer 12V</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ABI-010-RC</t>
+    <t xml:space="preserve">NA555P</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Buzzer (6 – 16V, 85dBA)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AT-1224-TWT-12V-R</t>
   </si>
   <si>
     <t xml:space="preserve">Schottky diode SOD 123</t>
@@ -88,10 +103,34 @@
     <t xml:space="preserve">MBR0520</t>
   </si>
   <si>
-    <t xml:space="preserve">Current fuses</t>
-  </si>
-  <si>
-    <t xml:space="preserve">MP005472</t>
+    <t xml:space="preserve">Schottky rectifier 100V/1A</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SS1H10-E3/5AT</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Tahoma"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">Current fuses </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Tahoma"/>
+        <family val="0"/>
+      </rPr>
+      <t xml:space="preserve"> 24V/10A</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">MP005472 (not important)</t>
   </si>
   <si>
     <t xml:space="preserve">DPS socket, CLIK-Mate 3 pin</t>
@@ -166,10 +205,10 @@
     <t xml:space="preserve">PE2512FKE070R01L</t>
   </si>
   <si>
-    <t xml:space="preserve">Resistor 200 805 5%</t>
-  </si>
-  <si>
-    <t xml:space="preserve">RC0805FR-07200RL</t>
+    <t xml:space="preserve">Resistor 110 805 1%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MCWR08X1100FTL</t>
   </si>
   <si>
     <t xml:space="preserve">Resistor 2k7 805 1%</t>
@@ -196,16 +235,22 @@
     <t xml:space="preserve">RC0805JR-10100KL</t>
   </si>
   <si>
-    <t xml:space="preserve">Resistor 590k 805 1%</t>
-  </si>
-  <si>
-    <t xml:space="preserve">RC0805FR-07590KL</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Capacitor 680pF 10% 805</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CC0805KRX7R9BB681</t>
+    <t xml:space="preserve">Resistor 560k 805 1%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MCWR08X564 JTL</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Resistor Network 10kohm</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MP000982</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Resistor Network 120ohm</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TC164-JR-07120RL</t>
   </si>
   <si>
     <t xml:space="preserve">Capacitor 0.1uF 10% 805</t>
@@ -214,34 +259,16 @@
     <t xml:space="preserve">CL21B104KBCNNND</t>
   </si>
   <si>
-    <t xml:space="preserve">Capacitor 220nF 10% 805</t>
-  </si>
-  <si>
-    <t xml:space="preserve">GRM21AR72A224KAC5K</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Capacitor 1uF 10% 805</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CL21B105KAFNNNE</t>
+    <t xml:space="preserve">Capacitor 0.33uF 10% 805</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CL21B334KBFNNNE</t>
   </si>
   <si>
     <t xml:space="preserve">Capacitor 10 uF 10% 805</t>
   </si>
   <si>
     <t xml:space="preserve">GRM21BC80J106KE19L</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Capacitor 22uF 10 % 805</t>
-  </si>
-  <si>
-    <t xml:space="preserve">GRM21BC80J226ME51L</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Capacitor 47uF 10% 805</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CL21A476MQCLRNC</t>
   </si>
 </sst>
 </file>
@@ -251,7 +278,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="General"/>
   </numFmts>
-  <fonts count="5">
+  <fonts count="7">
     <font>
       <sz val="10"/>
       <color theme="1"/>
@@ -281,6 +308,18 @@
       <name val="Tahoma"/>
       <family val="0"/>
       <charset val="1"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Nimbus Roman"/>
+      <family val="1"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Tahoma"/>
+      <family val="0"/>
     </font>
   </fonts>
   <fills count="2">
@@ -325,7 +364,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="9">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -336,6 +375,30 @@
     </xf>
     <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
@@ -534,7 +597,9 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="9"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="41.06"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="32.29"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="26" min="5" style="1" width="8.43"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="12.71"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="16.8"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="26" min="7" style="1" width="8.43"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -547,8 +612,12 @@
       <c r="C1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="2"/>
-      <c r="E1" s="2"/>
+      <c r="D1" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>4</v>
+      </c>
       <c r="F1" s="2"/>
       <c r="G1" s="2"/>
       <c r="H1" s="2"/>
@@ -579,10 +648,13 @@
         <v>5</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>4</v>
+        <v>6</v>
+      </c>
+      <c r="E2" s="1" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -593,10 +665,13 @@
         <v>5</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="D3" s="1" t="n">
+        <v>7</v>
+      </c>
+      <c r="D3" s="3" t="n">
         <v>104020006</v>
+      </c>
+      <c r="E3" s="1" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -607,38 +682,50 @@
         <v>5</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>7</v>
+        <v>9</v>
+      </c>
+      <c r="E4" s="1" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="1" t="n">
+      <c r="A5" s="4" t="n">
         <v>3007429</v>
       </c>
       <c r="B5" s="1" t="n">
         <v>5</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>9</v>
+        <v>11</v>
+      </c>
+      <c r="E5" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="F5" s="1" t="s">
+        <v>12</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="1" t="n">
+      <c r="A6" s="5" t="n">
         <v>3404609</v>
       </c>
       <c r="B6" s="1" t="n">
         <v>5</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>11</v>
+        <v>14</v>
+      </c>
+      <c r="E6" s="1" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -649,430 +736,523 @@
         <v>5</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>13</v>
+        <v>16</v>
+      </c>
+      <c r="E7" s="1" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="1" t="n">
+      <c r="A8" s="5" t="n">
         <v>3589297</v>
       </c>
       <c r="B8" s="1" t="n">
         <v>5</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>15</v>
+        <v>18</v>
+      </c>
+      <c r="E8" s="1" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="1" t="n">
-        <v>3121177</v>
-      </c>
-      <c r="B9" s="1" t="n">
+      <c r="A9" s="5" t="n">
+        <v>4294840</v>
+      </c>
+      <c r="B9" s="0" t="n">
         <v>5</v>
       </c>
-      <c r="C9" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="D9" s="1" t="s">
-        <v>17</v>
+      <c r="C9" s="0" t="s">
+        <v>19</v>
+      </c>
+      <c r="D9" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="E9" s="0" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="1" t="n">
-        <v>1022399</v>
+        <v>3121189</v>
       </c>
       <c r="B10" s="1" t="n">
         <v>5</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>19</v>
+        <v>22</v>
+      </c>
+      <c r="E10" s="1" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="1" t="n">
-        <v>2533224</v>
+      <c r="A11" s="6" t="n">
+        <v>4411167</v>
       </c>
       <c r="B11" s="1" t="n">
         <v>5</v>
       </c>
-      <c r="C11" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="D11" s="1" t="s">
-        <v>21</v>
+      <c r="C11" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="D11" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="E11" s="1" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="1" t="n">
-        <v>3564732</v>
+        <v>2533224</v>
       </c>
       <c r="B12" s="1" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="D12" s="1" t="s">
-        <v>23</v>
+        <v>26</v>
+      </c>
+      <c r="E12" s="1" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="1" t="n">
-        <v>2914017</v>
+        <v>2889241</v>
       </c>
       <c r="B13" s="1" t="n">
         <v>5</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="D13" s="1" t="s">
-        <v>25</v>
+        <v>28</v>
+      </c>
+      <c r="E13" s="1" t="n">
+        <v>3</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="1" t="n">
-        <v>1617068</v>
+        <v>3564732</v>
       </c>
       <c r="B14" s="1" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="D14" s="1" t="s">
-        <v>27</v>
+        <v>30</v>
+      </c>
+      <c r="E14" s="1" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="1" t="n">
-        <v>3221826</v>
+        <v>2914017</v>
       </c>
       <c r="B15" s="1" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="D15" s="1" t="s">
-        <v>29</v>
+        <v>32</v>
+      </c>
+      <c r="E15" s="1" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="1" t="n">
-        <v>2913997</v>
+        <v>1617068</v>
       </c>
       <c r="B16" s="1" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="D16" s="1" t="s">
-        <v>31</v>
+        <v>34</v>
+      </c>
+      <c r="E16" s="1" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="1" t="n">
-        <v>1617057</v>
+        <v>3221826</v>
       </c>
       <c r="B17" s="1" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="D17" s="1" t="s">
-        <v>33</v>
+        <v>36</v>
+      </c>
+      <c r="E17" s="1" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="1" t="n">
-        <v>3864009</v>
+        <v>2913997</v>
       </c>
       <c r="B18" s="1" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>34</v>
+        <v>37</v>
       </c>
       <c r="D18" s="1" t="s">
-        <v>35</v>
+        <v>38</v>
+      </c>
+      <c r="E18" s="1" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="1" t="n">
+        <v>1617057</v>
+      </c>
+      <c r="B19" s="1" t="n">
+        <v>10</v>
+      </c>
+      <c r="C19" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="D19" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="E19" s="1" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A20" s="6" t="n">
+        <v>3864009</v>
+      </c>
+      <c r="B20" s="1" t="n">
+        <v>10</v>
+      </c>
+      <c r="C20" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="D20" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="E20" s="1" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A21" s="6" t="n">
         <v>2313700</v>
       </c>
-      <c r="B19" s="1" t="n">
-        <v>100</v>
-      </c>
-      <c r="C19" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="D19" s="1" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="20" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="1" t="n">
+      <c r="B21" s="1" t="n">
+        <v>20</v>
+      </c>
+      <c r="C21" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="D21" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="E21" s="1" t="n">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A22" s="6" t="n">
         <v>2530074</v>
-      </c>
-      <c r="B20" s="1" t="n">
-        <v>5</v>
-      </c>
-      <c r="C20" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="D20" s="1" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="21" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A21" s="1" t="n">
-        <v>4553395</v>
-      </c>
-      <c r="B21" s="1" t="n">
-        <v>5</v>
-      </c>
-      <c r="C21" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="D21" s="1" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="22" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A22" s="1" t="n">
-        <v>3772839</v>
       </c>
       <c r="B22" s="1" t="n">
         <v>5</v>
       </c>
       <c r="C22" s="1" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="D22" s="1" t="s">
-        <v>43</v>
+        <v>46</v>
+      </c>
+      <c r="E22" s="1" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A23" s="1" t="n">
+      <c r="A23" s="6" t="n">
+        <v>4553395</v>
+      </c>
+      <c r="B23" s="1" t="n">
+        <v>5</v>
+      </c>
+      <c r="C23" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="D23" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="E23" s="1" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A24" s="6" t="n">
+        <v>3772839</v>
+      </c>
+      <c r="B24" s="1" t="n">
+        <v>5</v>
+      </c>
+      <c r="C24" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="D24" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="E24" s="1" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A25" s="6" t="n">
         <v>2309112</v>
-      </c>
-      <c r="B23" s="1" t="n">
-        <v>40</v>
-      </c>
-      <c r="C23" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="D23" s="1" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="24" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A24" s="1" t="n">
-        <v>3951690</v>
-      </c>
-      <c r="B24" s="1" t="n">
-        <v>10</v>
-      </c>
-      <c r="C24" s="1" t="s">
-        <v>46</v>
-      </c>
-      <c r="D24" s="1" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="25" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A25" s="1" t="n">
-        <v>3495998</v>
       </c>
       <c r="B25" s="1" t="n">
         <v>10</v>
       </c>
       <c r="C25" s="1" t="s">
-        <v>48</v>
+        <v>51</v>
       </c>
       <c r="D25" s="1" t="s">
-        <v>49</v>
+        <v>52</v>
+      </c>
+      <c r="E25" s="1" t="n">
+        <v>5</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A26" s="1" t="n">
-        <v>9237666</v>
+      <c r="A26" s="6" t="n">
+        <v>3951690</v>
       </c>
       <c r="B26" s="1" t="n">
         <v>10</v>
       </c>
       <c r="C26" s="1" t="s">
-        <v>50</v>
+        <v>53</v>
       </c>
       <c r="D26" s="1" t="s">
-        <v>51</v>
+        <v>54</v>
+      </c>
+      <c r="E26" s="1" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A27" s="1" t="n">
-        <v>3496134</v>
+      <c r="A27" s="5" t="n">
+        <v>2447558</v>
       </c>
       <c r="B27" s="1" t="n">
         <v>10</v>
       </c>
       <c r="C27" s="1" t="s">
-        <v>52</v>
-      </c>
-      <c r="D27" s="1" t="s">
-        <v>53</v>
+        <v>55</v>
+      </c>
+      <c r="D27" s="0" t="s">
+        <v>56</v>
+      </c>
+      <c r="E27" s="1" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="1" t="n">
-        <v>4139748</v>
+        <v>9237666</v>
       </c>
       <c r="B28" s="1" t="n">
-        <v>40</v>
+        <v>10</v>
       </c>
       <c r="C28" s="1" t="s">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="D28" s="1" t="s">
-        <v>55</v>
+        <v>58</v>
+      </c>
+      <c r="E28" s="1" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="1" t="n">
-        <v>4013422</v>
+        <v>3496134</v>
       </c>
       <c r="B29" s="1" t="n">
         <v>10</v>
       </c>
       <c r="C29" s="1" t="s">
-        <v>56</v>
+        <v>59</v>
       </c>
       <c r="D29" s="1" t="s">
-        <v>57</v>
+        <v>60</v>
+      </c>
+      <c r="E29" s="1" t="n">
+        <v>10</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A30" s="1" t="n">
-        <v>3952338</v>
+        <v>4139748</v>
       </c>
       <c r="B30" s="1" t="n">
         <v>10</v>
       </c>
       <c r="C30" s="1" t="s">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="D30" s="1" t="s">
-        <v>59</v>
+        <v>62</v>
+      </c>
+      <c r="E30" s="1" t="n">
+        <v>6</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A31" s="1" t="n">
-        <v>3019860</v>
+        <v>4013422</v>
       </c>
       <c r="B31" s="1" t="n">
         <v>10</v>
       </c>
       <c r="C31" s="1" t="s">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="D31" s="1" t="s">
-        <v>61</v>
+        <v>64</v>
+      </c>
+      <c r="E31" s="1" t="n">
+        <v>3</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A32" s="1" t="n">
-        <v>4539029</v>
+        <v>2695075</v>
       </c>
       <c r="B32" s="1" t="n">
         <v>10</v>
       </c>
       <c r="C32" s="1" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="D32" s="1" t="s">
-        <v>63</v>
+        <v>66</v>
+      </c>
+      <c r="E32" s="1" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A33" s="1" t="n">
-        <v>3785973</v>
+      <c r="A33" s="7" t="n">
+        <v>3228729</v>
       </c>
       <c r="B33" s="1" t="n">
         <v>10</v>
       </c>
       <c r="C33" s="1" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="D33" s="1" t="s">
-        <v>65</v>
+        <v>68</v>
+      </c>
+      <c r="E33" s="1" t="n">
+        <v>3</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A34" s="1" t="n">
-        <v>3013481</v>
+      <c r="A34" s="8" t="n">
+        <v>9235000</v>
       </c>
       <c r="B34" s="1" t="n">
         <v>10</v>
       </c>
       <c r="C34" s="1" t="s">
-        <v>66</v>
-      </c>
-      <c r="D34" s="1" t="s">
-        <v>67</v>
+        <v>69</v>
+      </c>
+      <c r="D34" s="5" t="s">
+        <v>70</v>
+      </c>
+      <c r="E34" s="1" t="n">
+        <v>1</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A35" s="1" t="n">
-        <v>4327048</v>
+        <v>4539029</v>
       </c>
       <c r="B35" s="1" t="n">
         <v>10</v>
       </c>
       <c r="C35" s="1" t="s">
-        <v>68</v>
+        <v>71</v>
       </c>
       <c r="D35" s="1" t="s">
-        <v>69</v>
+        <v>72</v>
+      </c>
+      <c r="E35" s="1" t="n">
+        <v>9</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A36" s="1" t="n">
-        <v>4361089</v>
+      <c r="A36" s="0" t="n">
+        <v>4539154</v>
       </c>
       <c r="B36" s="1" t="n">
         <v>10</v>
       </c>
       <c r="C36" s="1" t="s">
-        <v>70</v>
-      </c>
-      <c r="D36" s="1" t="s">
-        <v>71</v>
+        <v>73</v>
+      </c>
+      <c r="D36" s="0" t="s">
+        <v>74</v>
+      </c>
+      <c r="E36" s="1" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A37" s="1" t="n">
-        <v>3013465</v>
+      <c r="A37" s="5" t="n">
+        <v>4327048</v>
       </c>
       <c r="B37" s="1" t="n">
         <v>10</v>
       </c>
       <c r="C37" s="1" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="D37" s="1" t="s">
-        <v>73</v>
+        <v>76</v>
+      </c>
+      <c r="E37" s="1" t="n">
+        <v>2</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>

</xml_diff>